<commit_message>
Pre-deployment cleanup: remove dead debug script and duplicate folder, gitignore app/ and app.zip, fix nginx basePath redirect for /Dashboard
</commit_message>
<xml_diff>
--- a/Input/OffDays.xlsx
+++ b/Input/OffDays.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\PowerBIData\Input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\07PREPORT\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21E93427-242F-4B36-9B0B-DC09D39CA03D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76A8CA46-2ABE-42CF-B06A-342A4A39A57B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{270FB6C7-A2B3-40AC-B073-E90C78E630F8}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="45">
   <si>
     <t>Date</t>
   </si>
@@ -74,9 +74,6 @@
     <t>Unexpected</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
     <t>official</t>
   </si>
   <si>
@@ -153,6 +150,30 @@
   </si>
   <si>
     <t>30/5/2026</t>
+  </si>
+  <si>
+    <t>عيد الفطر</t>
+  </si>
+  <si>
+    <t>عيد العمال</t>
+  </si>
+  <si>
+    <t>عيد الاضحى</t>
+  </si>
+  <si>
+    <t>عيد الميلود</t>
+  </si>
+  <si>
+    <t>عاصفة</t>
+  </si>
+  <si>
+    <t>طريق مغلق</t>
+  </si>
+  <si>
+    <t>سرقة</t>
+  </si>
+  <si>
+    <t>اضطرارية</t>
   </si>
 </sst>
 </file>
@@ -583,10 +604,10 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>5</v>
@@ -600,23 +621,25 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" s="4"/>
+        <v>44</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>43</v>
+      </c>
       <c r="E2" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F2" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="G2" s="6" t="s">
         <v>24</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>25</v>
       </c>
       <c r="H2" s="2">
         <v>1</v>
@@ -628,23 +651,25 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="4"/>
+        <v>44</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="E3" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" s="6" t="s">
         <v>24</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>25</v>
       </c>
       <c r="H3" s="2">
         <v>1</v>
@@ -656,23 +681,25 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="4"/>
+        <v>44</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="E4" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H4" s="2">
         <v>1</v>
@@ -684,23 +711,25 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="4"/>
+        <v>44</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="E5" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H5" s="2">
         <v>1</v>
@@ -712,23 +741,25 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="4"/>
+        <v>44</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="E6" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H6" s="2">
         <v>1</v>
@@ -740,23 +771,25 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>10</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="4"/>
+        <v>44</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="E7" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H7" s="2">
         <v>1</v>
@@ -768,10 +801,13 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>37</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>8</v>
@@ -785,10 +821,13 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>37</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>8</v>
@@ -802,10 +841,13 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>37</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>8</v>
@@ -819,10 +861,13 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>37</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>8</v>
@@ -839,7 +884,10 @@
         <v>46143</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>38</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>8</v>
@@ -853,10 +901,13 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>39</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>8</v>
@@ -870,10 +921,13 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>39</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>8</v>
@@ -887,10 +941,13 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>39</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>8</v>
@@ -904,10 +961,13 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>39</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>8</v>
@@ -921,10 +981,13 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>40</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>8</v>
@@ -938,10 +1001,13 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>40</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>8</v>
@@ -960,14 +1026,20 @@
       <c r="B19" s="4" t="s">
         <v>10</v>
       </c>
+      <c r="C19" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D19" t="s">
+        <v>42</v>
+      </c>
       <c r="E19" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H19" s="2">
         <v>1</v>
@@ -978,19 +1050,25 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>10</v>
       </c>
+      <c r="C20" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D20" t="s">
+        <v>42</v>
+      </c>
       <c r="E20" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H20" s="2">
         <v>1</v>
@@ -1001,19 +1079,25 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>10</v>
       </c>
+      <c r="C21" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D21" t="s">
+        <v>42</v>
+      </c>
       <c r="E21" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H21" s="2">
         <v>1</v>
@@ -1024,19 +1108,25 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>10</v>
       </c>
+      <c r="C22" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D22" t="s">
+        <v>42</v>
+      </c>
       <c r="E22" s="4" t="s">
         <v>8</v>
       </c>
       <c r="F22" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="G22" s="6" t="s">
         <v>24</v>
-      </c>
-      <c r="G22" s="6" t="s">
-        <v>25</v>
       </c>
       <c r="H22" s="2">
         <v>1</v>

</xml_diff>